<commit_message>
Changed PLAPD to PLPD
</commit_message>
<xml_diff>
--- a/Data/2023_F013B4_CO_TILL/2023_F013B4_CO_TILL_CropCanopy.xlsx
+++ b/Data/2023_F013B4_CO_TILL/2023_F013B4_CO_TILL_CropCanopy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\mnt\Data1\USDA-ALARC\GIS\PDI project\cottondata\Data\2023_F013B4_CO_TILL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{728C4A64-2481-4704-818E-0E408A03FFFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D4711FB-CBF3-41C4-93EF-3EAF98C4F007}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16455" yWindow="-28440" windowWidth="17805" windowHeight="11445" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-1470" yWindow="-25290" windowWidth="17805" windowHeight="20370" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Height" sheetId="12" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3487" uniqueCount="504">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3487" uniqueCount="505">
   <si>
     <t>01-</t>
   </si>
@@ -1607,6 +1607,9 @@
   <si>
     <t>date:</t>
   </si>
+  <si>
+    <t>PLPD</t>
+  </si>
 </sst>
 </file>
 
@@ -3113,7 +3116,25 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="21" fillId="0" borderId="35" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="167" fontId="19" fillId="0" borderId="32" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="19" fillId="0" borderId="8" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="2" fillId="0" borderId="38" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -3122,28 +3143,10 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="3" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="21" fillId="0" borderId="37" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="21" fillId="0" borderId="35" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="19" fillId="0" borderId="8" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -17651,33 +17654,33 @@
       <c r="C11" s="186" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="227">
+      <c r="D11" s="232">
         <v>45048</v>
       </c>
-      <c r="E11" s="228"/>
-      <c r="F11" s="227">
+      <c r="E11" s="234"/>
+      <c r="F11" s="232">
         <v>45050</v>
       </c>
-      <c r="G11" s="228"/>
-      <c r="H11" s="227">
+      <c r="G11" s="234"/>
+      <c r="H11" s="232">
         <v>45054</v>
       </c>
-      <c r="I11" s="228"/>
-      <c r="J11" s="227">
+      <c r="I11" s="234"/>
+      <c r="J11" s="232">
         <v>45057</v>
       </c>
-      <c r="K11" s="236"/>
-      <c r="L11" s="228"/>
-      <c r="M11" s="227">
+      <c r="K11" s="233"/>
+      <c r="L11" s="234"/>
+      <c r="M11" s="232">
         <v>45061</v>
       </c>
-      <c r="N11" s="236"/>
-      <c r="O11" s="228"/>
-      <c r="P11" s="227">
+      <c r="N11" s="233"/>
+      <c r="O11" s="234"/>
+      <c r="P11" s="232">
         <v>45064</v>
       </c>
-      <c r="Q11" s="236"/>
-      <c r="R11" s="228"/>
+      <c r="Q11" s="233"/>
+      <c r="R11" s="234"/>
     </row>
     <row r="12" spans="1:18" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="184" t="s">
@@ -17686,33 +17689,33 @@
       <c r="C12" s="183" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="229">
+      <c r="D12" s="235">
         <v>122</v>
       </c>
-      <c r="E12" s="230"/>
-      <c r="F12" s="229">
+      <c r="E12" s="229"/>
+      <c r="F12" s="235">
         <v>124</v>
       </c>
-      <c r="G12" s="230"/>
-      <c r="H12" s="229">
+      <c r="G12" s="229"/>
+      <c r="H12" s="235">
         <v>128</v>
       </c>
-      <c r="I12" s="230"/>
-      <c r="J12" s="229">
+      <c r="I12" s="229"/>
+      <c r="J12" s="235">
         <v>131</v>
       </c>
-      <c r="K12" s="237"/>
-      <c r="L12" s="230"/>
-      <c r="M12" s="229">
+      <c r="K12" s="236"/>
+      <c r="L12" s="229"/>
+      <c r="M12" s="235">
         <v>135</v>
       </c>
-      <c r="N12" s="237"/>
-      <c r="O12" s="230"/>
-      <c r="P12" s="229">
+      <c r="N12" s="236"/>
+      <c r="O12" s="229"/>
+      <c r="P12" s="235">
         <v>138</v>
       </c>
-      <c r="Q12" s="237"/>
-      <c r="R12" s="230"/>
+      <c r="Q12" s="236"/>
+      <c r="R12" s="229"/>
     </row>
     <row r="13" spans="1:18" s="178" customFormat="1" ht="28.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="181" t="s">
@@ -17721,50 +17724,50 @@
       <c r="C13" s="180" t="s">
         <v>9</v>
       </c>
-      <c r="D13" s="233" t="s">
+      <c r="D13" s="227" t="s">
         <v>458</v>
       </c>
-      <c r="E13" s="230"/>
-      <c r="F13" s="233" t="s">
+      <c r="E13" s="229"/>
+      <c r="F13" s="227" t="s">
         <v>457</v>
       </c>
-      <c r="G13" s="230"/>
-      <c r="H13" s="233" t="s">
+      <c r="G13" s="229"/>
+      <c r="H13" s="227" t="s">
         <v>456</v>
       </c>
-      <c r="I13" s="230"/>
-      <c r="J13" s="233" t="s">
+      <c r="I13" s="229"/>
+      <c r="J13" s="227" t="s">
         <v>455</v>
       </c>
-      <c r="K13" s="235"/>
-      <c r="L13" s="230"/>
-      <c r="M13" s="233" t="s">
+      <c r="K13" s="228"/>
+      <c r="L13" s="229"/>
+      <c r="M13" s="227" t="s">
         <v>454</v>
       </c>
-      <c r="N13" s="235"/>
-      <c r="O13" s="230"/>
-      <c r="P13" s="233" t="s">
+      <c r="N13" s="228"/>
+      <c r="O13" s="229"/>
+      <c r="P13" s="227" t="s">
         <v>453</v>
       </c>
-      <c r="Q13" s="235"/>
-      <c r="R13" s="230"/>
+      <c r="Q13" s="228"/>
+      <c r="R13" s="229"/>
     </row>
     <row r="14" spans="1:18" s="131" customFormat="1" ht="8.4499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="174"/>
       <c r="B14" s="173"/>
       <c r="C14" s="172"/>
-      <c r="D14" s="231"/>
-      <c r="E14" s="232"/>
-      <c r="F14" s="234"/>
-      <c r="G14" s="232"/>
-      <c r="H14" s="234"/>
-      <c r="I14" s="232"/>
-      <c r="J14" s="234"/>
-      <c r="K14" s="234"/>
-      <c r="L14" s="232"/>
-      <c r="M14" s="234"/>
-      <c r="N14" s="234"/>
-      <c r="O14" s="232"/>
+      <c r="D14" s="237"/>
+      <c r="E14" s="231"/>
+      <c r="F14" s="230"/>
+      <c r="G14" s="231"/>
+      <c r="H14" s="230"/>
+      <c r="I14" s="231"/>
+      <c r="J14" s="230"/>
+      <c r="K14" s="230"/>
+      <c r="L14" s="231"/>
+      <c r="M14" s="230"/>
+      <c r="N14" s="230"/>
+      <c r="O14" s="231"/>
       <c r="P14" s="176"/>
       <c r="Q14" s="176"/>
       <c r="R14" s="175"/>
@@ -27011,6 +27014,18 @@
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H14:I14"/>
     <mergeCell ref="J13:L13"/>
     <mergeCell ref="M14:O14"/>
     <mergeCell ref="J14:L14"/>
@@ -27022,18 +27037,6 @@
     <mergeCell ref="P13:R13"/>
     <mergeCell ref="J11:L11"/>
     <mergeCell ref="J12:L12"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="H12:I12"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0" footer="0.25"/>
@@ -27179,7 +27182,7 @@
         <v>8</v>
       </c>
       <c r="I4" s="130">
-        <f t="shared" ref="I3:I34" si="0">H4/2</f>
+        <f t="shared" ref="I4:I34" si="0">H4/2</f>
         <v>4</v>
       </c>
       <c r="J4" s="134">
@@ -49818,7 +49821,7 @@
         <v>414</v>
       </c>
       <c r="B1" s="127" t="s">
-        <v>423</v>
+        <v>504</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>